<commit_message>
feat: release v1.2.0 with reachable architecture and pipeline pages
Tighten W% to a 20-60% colocation ladder, add mermaid/YAML tabs with keyboard and skip-link access, and publish the standalone HTML so GitHub Pages serves the live planner.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/dist/CICD_Tool_Resource_Matrix.xlsx
+++ b/dist/CICD_Tool_Resource_Matrix.xlsx
@@ -2765,7 +2765,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 — ใช้เป็นแบบฟอร์มกลางสำหรับประเมินโครงการใด ๆ (ไม่มีข้อมูลเฉพาะโครงการอยู่ในไฟล์นี้)</t>
+          <t>Schema 1.2.0 — ใช้เป็นแบบฟอร์มกลางสำหรับประเมินโครงการใด ๆ (ไม่มีข้อมูลเฉพาะโครงการอยู่ในไฟล์นี้)</t>
         </is>
       </c>
     </row>
@@ -3632,10 +3632,10 @@
         <v>7</v>
       </c>
       <c r="F3" s="136" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G3" s="136" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H3" s="136" t="n">
         <v>200</v>
@@ -3666,10 +3666,10 @@
         <v>24</v>
       </c>
       <c r="F4" s="136" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G4" s="136" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="H4" s="136" t="n">
         <v>1000</v>
@@ -3695,10 +3695,10 @@
         </is>
       </c>
       <c r="F5" s="139" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="G5" s="139" t="n">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="H5" s="139" t="n">
         <v>1200</v>
@@ -3732,10 +3732,10 @@
         <v>9</v>
       </c>
       <c r="F7" s="143" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G7" s="143" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="H7" s="143" t="n">
         <v>300</v>
@@ -3766,10 +3766,10 @@
         <v>21</v>
       </c>
       <c r="F8" s="143" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="143" t="n">
         <v>12</v>
-      </c>
-      <c r="G8" s="143" t="n">
-        <v>24</v>
       </c>
       <c r="H8" s="143" t="n">
         <v>750</v>
@@ -3800,10 +3800,10 @@
         <v>8</v>
       </c>
       <c r="F9" s="143" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G9" s="143" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="H9" s="143" t="n">
         <v>300</v>
@@ -3834,10 +3834,10 @@
         <v>8</v>
       </c>
       <c r="F10" s="143" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G10" s="143" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H10" s="143" t="n">
         <v>300</v>
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="F11" s="139" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="G11" s="139" t="n">
-        <v>112</v>
+        <v>36</v>
       </c>
       <c r="H11" s="139" t="n">
         <v>1650</v>
@@ -3900,10 +3900,10 @@
         <v>4</v>
       </c>
       <c r="F13" s="136" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="136" t="n">
         <v>8</v>
-      </c>
-      <c r="G13" s="136" t="n">
-        <v>12</v>
       </c>
       <c r="H13" s="136" t="n">
         <v>100</v>
@@ -3934,10 +3934,10 @@
         <v>6</v>
       </c>
       <c r="F14" s="136" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G14" s="136" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H14" s="136" t="n">
         <v>150</v>
@@ -3968,10 +3968,10 @@
         <v>14</v>
       </c>
       <c r="F15" s="136" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G15" s="136" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H15" s="136" t="n">
         <v>500</v>
@@ -4036,10 +4036,10 @@
         <v>8</v>
       </c>
       <c r="F17" s="136" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G17" s="136" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="H17" s="136" t="n">
         <v>300</v>
@@ -4070,10 +4070,10 @@
         <v>8</v>
       </c>
       <c r="F18" s="136" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G18" s="136" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H18" s="136" t="n">
         <v>300</v>
@@ -4099,10 +4099,10 @@
         </is>
       </c>
       <c r="F19" s="139" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="G19" s="139" t="n">
-        <v>120</v>
+        <v>56</v>
       </c>
       <c r="H19" s="139" t="n">
         <v>1550</v>
@@ -4136,10 +4136,10 @@
         <v>8</v>
       </c>
       <c r="F21" s="143" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G21" s="143" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H21" s="143" t="n">
         <v>200</v>
@@ -4170,10 +4170,10 @@
         <v>19</v>
       </c>
       <c r="F22" s="143" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="143" t="n">
         <v>12</v>
-      </c>
-      <c r="G22" s="143" t="n">
-        <v>24</v>
       </c>
       <c r="H22" s="143" t="n">
         <v>750</v>
@@ -4204,10 +4204,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="143" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G23" s="143" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H23" s="143" t="n">
         <v>300</v>
@@ -4272,10 +4272,10 @@
         <v>8</v>
       </c>
       <c r="F25" s="143" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G25" s="143" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H25" s="143" t="n">
         <v>300</v>
@@ -4301,10 +4301,10 @@
         </is>
       </c>
       <c r="F26" s="139" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="G26" s="139" t="n">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="H26" s="139" t="n">
         <v>1850</v>
@@ -20529,7 +20529,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>w = w_base + w_span x activity_index  -&gt;  อยู่ในช่วง 50% - 95% ตามโจทย์</t>
+          <t>w_solo = w_base + w_span x activity_index  -&gt;  ช่วงเดี่ยว 20% - 60%; บน VM ใช้ w_max(n) ladder</t>
         </is>
       </c>
     </row>
@@ -20590,7 +20590,7 @@
       </c>
       <c r="F3" s="48" t="inlineStr">
         <is>
-          <t>กินหน่วยความจำถาวร เช่น Jenkins Master, Elasticsearch, PostgreSQL, MinIO — บวกเต็มเกือบ 100%</t>
+          <t>น้ำหนักสูงสุด 60% เมื่ออยู่เครื่องเดียว ลดตามจำนวนเครื่องมือร่วมเครื่องลงถึงพื้น 20%</t>
         </is>
       </c>
     </row>
@@ -20619,7 +20619,7 @@
       </c>
       <c r="F4" s="48" t="inlineStr">
         <is>
-          <t>Trigger บ่อยมาก เกิดการซ้อนทับของงาน (overlap) สูง</t>
+          <t>Trigger บ่อย ยังซ้อนทับได้ แต่ถูกจำกัดด้วยเพดาน w_max(n) ของเครื่องนั้น</t>
         </is>
       </c>
     </row>
@@ -20764,14 +20764,14 @@
       </c>
       <c r="F9" s="48" t="inlineStr">
         <is>
-          <t>บวกที่ 50% ซึ่งเป็นค่าต่ำสุดของช่วงที่กำหนด เพราะยังต้องกันที่ไว้ให้รันได้</t>
+          <t>บวกที่ 20% ซึ่งเป็นค่าต่ำสุดของช่วงที่กำหนด เพราะยังต้องกันที่ไว้ให้รันได้</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>ที่มาของช่วง 50-95%: เป็นเงื่อนไขที่กำหนดในโจทย์ — เครื่องมือที่รันตามคำสั่ง/รอบ Release บวกที่ 50% (ยังต้องกันที่ไว้ให้รันได้) ส่วนเครื่องมือที่รันค้าง 24/7 บวกที่ 95% (เกือบเต็มเพราะจองหน่วยความจำถาวร)</t>
+          <t>ช่วง 20-60%: เครื่องมือตามคำสั่งบวกที่ 20% (กันที่ไว้ให้รันได้) เครื่องมือ resident บนเครื่องเดียวบวกที่ 60% แล้วลดตามจำนวนเครื่องมือร่วมเครื่อง ลงถึงพื้น 20% เมื่อมี 8 ตัวขึ้นไป</t>
         </is>
       </c>
     </row>
@@ -30266,11 +30266,11 @@
         </is>
       </c>
       <c r="B9" s="90" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="C9" s="91" t="inlineStr">
         <is>
-          <t>คือ 50% ตามโจทย์ที่กำหนด — ใช้กับเครื่องมือที่รันตามคำสั่ง/รอบ Release</t>
+          <t>คือ 20% — ใช้กับเครื่องมือที่รันตามคำสั่ง/รอบ Release</t>
         </is>
       </c>
       <c r="E9" s="93" t="n">
@@ -30290,11 +30290,11 @@
         </is>
       </c>
       <c r="B10" s="90" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="C10" s="91" t="inlineStr">
         <is>
-          <t>คือ 0.45 ทำให้น้ำหนักสูงสุด = 0.50 + 0.45 = 0.95 (95%) ตามโจทย์</t>
+          <t>คือ 0.40 ทำให้น้ำหนักเดี่ยวสูงสุด = 0.20 + 0.40 = 0.60 (60%) เมื่ออยู่เครื่องเดียว</t>
         </is>
       </c>
       <c r="E10" s="93" t="n">

</xml_diff>